<commit_message>
feature/fsel-4792: update learning progress api
</commit_message>
<xml_diff>
--- a/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportLearningSchoolEvent.xlsx
+++ b/Services/Fsel.Course/Fsel.Course.Lms.Api/Resources/ExportExcelTemplates/ReportLearningSchoolEvent.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Backend\fsel_src\Services\Fsel.Course\Fsel.Course.Lms.Api\Resources\ExportExcelTemplates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3820375-1330-4678-9223-AE6E52EC91C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EB582DB-7EEC-4564-AD04-27E05ACB5658}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-135" windowWidth="29040" windowHeight="15720" xr2:uid="{CE6DB55D-6F3C-4AEA-8AE1-893538C51C25}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CE6DB55D-6F3C-4AEA-8AE1-893538C51C25}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="20">
   <si>
     <t>STT</t>
   </si>
@@ -78,7 +78,13 @@
     <t>[{0}] SỐ LIỆU ĐĂNG KÝ &amp; TIẾN TRÌNH HỌC TẬP TRÊN FSEL</t>
   </si>
   <si>
-    <t>học chương trình [{0}]</t>
+    <t>chọn chương trình [{0}]</t>
+  </si>
+  <si>
+    <t>tham gia học chương trình [{0}]</t>
+  </si>
+  <si>
+    <t>Quận/ Huyện</t>
   </si>
 </sst>
 </file>
@@ -337,7 +343,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -394,6 +400,19 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -710,13 +729,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09929B56-84AE-4290-93FF-52994429D500}">
-  <dimension ref="A2:R5"/>
+  <dimension ref="A2:T5"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="6" width="13.875" customWidth="1"/>
+    <col min="2" max="2" width="9" style="20"/>
+    <col min="3" max="8" width="13.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:18" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:20" ht="15.75" x14ac:dyDescent="0.2">
       <c r="A2" s="6" t="s">
         <v>16</v>
       </c>
@@ -737,31 +757,37 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
       <c r="R2" s="7"/>
+      <c r="S2" s="7"/>
+      <c r="T2" s="7"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A3" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="11" t="s">
+      <c r="B3" s="22" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>1</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>2</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="G3" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G3" s="14" t="s">
+      <c r="H3" s="21" t="s">
+        <v>2</v>
+      </c>
+      <c r="I3" s="14" t="s">
         <v>9</v>
       </c>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
       <c r="J3" s="15"/>
       <c r="K3" s="15"/>
       <c r="L3" s="15"/>
@@ -770,28 +796,32 @@
       <c r="O3" s="15"/>
       <c r="P3" s="15"/>
       <c r="Q3" s="15"/>
-      <c r="R3" s="16"/>
+      <c r="R3" s="15"/>
+      <c r="S3" s="15"/>
+      <c r="T3" s="16"/>
     </row>
-    <row r="4" spans="1:18" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:20" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="9"/>
-      <c r="B4" s="12"/>
-      <c r="C4" s="4" t="s">
+      <c r="B4" s="23"/>
+      <c r="C4" s="12"/>
+      <c r="D4" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="E4" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="F4" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="G4" s="17" t="s">
+      <c r="H4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="17" t="s">
         <v>7</v>
       </c>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
       <c r="J4" s="18"/>
       <c r="K4" s="18"/>
       <c r="L4" s="18"/>
@@ -800,63 +830,69 @@
       <c r="O4" s="18"/>
       <c r="P4" s="18"/>
       <c r="Q4" s="18"/>
-      <c r="R4" s="19"/>
+      <c r="R4" s="18"/>
+      <c r="S4" s="18"/>
+      <c r="T4" s="19"/>
     </row>
-    <row r="5" spans="1:18" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:20" ht="29.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="10"/>
-      <c r="B5" s="13"/>
-      <c r="C5" s="5"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="13"/>
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
       <c r="F5" s="5"/>
-      <c r="G5" s="2" t="s">
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+      <c r="I5" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="H5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>11</v>
       </c>
       <c r="J5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P5" s="2" t="s">
         <v>8</v>
       </c>
       <c r="Q5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="S5" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="R5" s="3" t="s">
+      <c r="T5" s="3" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="F4:F5"/>
-    <mergeCell ref="A2:R2"/>
+  <mergeCells count="11">
+    <mergeCell ref="G4:G5"/>
+    <mergeCell ref="A2:T2"/>
     <mergeCell ref="A3:A5"/>
-    <mergeCell ref="B3:B5"/>
-    <mergeCell ref="G3:R3"/>
-    <mergeCell ref="G4:R4"/>
-    <mergeCell ref="C4:C5"/>
+    <mergeCell ref="C3:C5"/>
+    <mergeCell ref="I3:T3"/>
+    <mergeCell ref="I4:T4"/>
     <mergeCell ref="D4:D5"/>
     <mergeCell ref="E4:E5"/>
+    <mergeCell ref="F4:F5"/>
+    <mergeCell ref="H4:H5"/>
+    <mergeCell ref="B3:B5"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>